<commit_message>
Update inventory via Laserax Inventory Manager
</commit_message>
<xml_diff>
--- a/Inventory.xlsx
+++ b/Inventory.xlsx
@@ -471,7 +471,11 @@
           <t>G1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>-</t>

</xml_diff>

<commit_message>
Update inventory via Streamlit
</commit_message>
<xml_diff>
--- a/Inventory.xlsx
+++ b/Inventory.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G153"/>
+  <dimension ref="A1:G154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3975,6 +3975,35 @@
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr"/>
     </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Coupling relay</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>PHOENIX 2903370 - RIF-0-RPT-24DC/21</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>12</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>G1(Storage)-B1</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Product No. 2961105</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>